<commit_message>
Fixed the svg layers save method, but there is a small issue with too many lines being drawn
</commit_message>
<xml_diff>
--- a/Materials.xlsx
+++ b/Materials.xlsx
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -150,9 +150,6 @@
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -478,9 +475,6 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11">
-      <c r="C11" s="6"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>